<commit_message>
ajustes nas mestas filiais 1,3 e PI
</commit_message>
<xml_diff>
--- a/data/meta_rca.xlsx
+++ b/data/meta_rca.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CADBA25-8F3C-4732-977F-6210CFF28A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5721B648-8418-44CA-A870-E46B8BCEA7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="2850" windowWidth="24240" windowHeight="13140" xr2:uid="{91476B03-704D-4E23-9E63-F1D303A50E23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{91476B03-704D-4E23-9E63-F1D303A50E23}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$C$386</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -452,7 +455,7 @@
         <v>42</v>
       </c>
       <c r="C2">
-        <v>248586.62882916722</v>
+        <v>290000</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -463,7 +466,7 @@
         <v>1064</v>
       </c>
       <c r="C3">
-        <v>172051.112835629</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -474,7 +477,7 @@
         <v>610</v>
       </c>
       <c r="C4">
-        <v>162731.03146504538</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -485,7 +488,7 @@
         <v>483</v>
       </c>
       <c r="C5">
-        <v>143993.04235115531</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -496,7 +499,7 @@
         <v>131</v>
       </c>
       <c r="C6">
-        <v>143595.53691699277</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -518,7 +521,7 @@
         <v>89</v>
       </c>
       <c r="C8">
-        <v>107002.35735440545</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -529,7 +532,7 @@
         <v>285</v>
       </c>
       <c r="C9">
-        <v>105839.46501357346</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -540,7 +543,7 @@
         <v>1075</v>
       </c>
       <c r="C10">
-        <v>104623.19037447221</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -551,7 +554,7 @@
         <v>953</v>
       </c>
       <c r="C11">
-        <v>99917.199831791586</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -562,7 +565,7 @@
         <v>1756</v>
       </c>
       <c r="C12">
-        <v>97572.09324418263</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -573,7 +576,7 @@
         <v>1117</v>
       </c>
       <c r="C13">
-        <v>96805.12638945764</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -584,7 +587,7 @@
         <v>1993</v>
       </c>
       <c r="C14">
-        <v>93967.008902712754</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -595,7 +598,7 @@
         <v>2250</v>
       </c>
       <c r="C15">
-        <v>91864.205755926363</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -606,7 +609,7 @@
         <v>629</v>
       </c>
       <c r="C16">
-        <v>81083.75968095717</v>
+        <v>115000</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -617,7 +620,7 @@
         <v>1465</v>
       </c>
       <c r="C17">
-        <v>79231.47255520802</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -628,7 +631,7 @@
         <v>619</v>
       </c>
       <c r="C18">
-        <v>69995.344925566329</v>
+        <v>64000</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -639,7 +642,7 @@
         <v>1063</v>
       </c>
       <c r="C19">
-        <v>68814.465893406508</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -650,7 +653,7 @@
         <v>58</v>
       </c>
       <c r="C20">
-        <v>66146.304844212456</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -661,7 +664,7 @@
         <v>40</v>
       </c>
       <c r="C21">
-        <v>56475.696175647339</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -672,7 +675,7 @@
         <v>451</v>
       </c>
       <c r="C22">
-        <v>55471.964497175686</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -683,7 +686,7 @@
         <v>1983</v>
       </c>
       <c r="C23">
-        <v>55403.569595082394</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -694,7 +697,7 @@
         <v>1478</v>
       </c>
       <c r="C24">
-        <v>52997.078968309223</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -705,7 +708,7 @@
         <v>1102</v>
       </c>
       <c r="C25">
-        <v>52928.337510386627</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -716,7 +719,7 @@
         <v>424</v>
       </c>
       <c r="C26">
-        <v>52633.525110919007</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -727,7 +730,7 @@
         <v>664</v>
       </c>
       <c r="C27">
-        <v>50402.60356501268</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -738,7 +741,7 @@
         <v>1937</v>
       </c>
       <c r="C28">
-        <v>50286.156844770187</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -749,7 +752,7 @@
         <v>559</v>
       </c>
       <c r="C29">
-        <v>47660.748549882264</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -760,7 +763,7 @@
         <v>530</v>
       </c>
       <c r="C30">
-        <v>43814.152962821179</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -771,7 +774,7 @@
         <v>2279</v>
       </c>
       <c r="C31">
-        <v>41527.363243473039</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -782,7 +785,7 @@
         <v>663</v>
       </c>
       <c r="C32">
-        <v>40734.237976708908</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -793,7 +796,7 @@
         <v>2251</v>
       </c>
       <c r="C33">
-        <v>38526.339324711858</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -804,7 +807,7 @@
         <v>1116</v>
       </c>
       <c r="C34">
-        <v>30124.720589466342</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -815,7 +818,7 @@
         <v>2245</v>
       </c>
       <c r="C35">
-        <v>28072.353694950514</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -826,7 +829,7 @@
         <v>477</v>
       </c>
       <c r="C36">
-        <v>27627.441166947752</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -837,7 +840,7 @@
         <v>2651</v>
       </c>
       <c r="C37">
-        <v>24680.411107499389</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -859,7 +862,7 @@
         <v>2463</v>
       </c>
       <c r="C39">
-        <v>17669.382940338797</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -1120,10 +1123,10 @@
         <v>3</v>
       </c>
       <c r="B63">
-        <v>2448</v>
+        <v>14</v>
       </c>
       <c r="C63">
-        <v>15000</v>
+        <v>114589.7365638465</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -1131,10 +1134,10 @@
         <v>3</v>
       </c>
       <c r="B64">
-        <v>2433</v>
+        <v>20</v>
       </c>
       <c r="C64">
-        <v>15000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
@@ -1142,7 +1145,7 @@
         <v>3</v>
       </c>
       <c r="B65">
-        <v>1658</v>
+        <v>27</v>
       </c>
       <c r="C65">
         <v>15000</v>
@@ -1153,10 +1156,10 @@
         <v>3</v>
       </c>
       <c r="B66">
-        <v>2588</v>
+        <v>33</v>
       </c>
       <c r="C66">
-        <v>15000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -1164,10 +1167,10 @@
         <v>3</v>
       </c>
       <c r="B67">
-        <v>783</v>
+        <v>104</v>
       </c>
       <c r="C67">
-        <v>15000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -1175,10 +1178,10 @@
         <v>3</v>
       </c>
       <c r="B68">
-        <v>802</v>
+        <v>132</v>
       </c>
       <c r="C68">
-        <v>15000</v>
+        <v>203686.51238615639</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -1208,10 +1211,10 @@
         <v>3</v>
       </c>
       <c r="B71">
-        <v>27</v>
+        <v>351</v>
       </c>
       <c r="C71">
-        <v>15000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -1219,10 +1222,10 @@
         <v>3</v>
       </c>
       <c r="B72">
-        <v>2440</v>
+        <v>400</v>
       </c>
       <c r="C72">
-        <v>15000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -1230,10 +1233,10 @@
         <v>3</v>
       </c>
       <c r="B73">
-        <v>1380</v>
+        <v>415</v>
       </c>
       <c r="C73">
-        <v>15000</v>
+        <v>123249.40959329615</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
@@ -1241,10 +1244,10 @@
         <v>3</v>
       </c>
       <c r="B74">
-        <v>400</v>
+        <v>438</v>
       </c>
       <c r="C74">
-        <v>15000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
@@ -1252,10 +1255,10 @@
         <v>3</v>
       </c>
       <c r="B75">
-        <v>580</v>
+        <v>452</v>
       </c>
       <c r="C75">
-        <v>15830.952946339548</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
@@ -1263,10 +1266,10 @@
         <v>3</v>
       </c>
       <c r="B76">
-        <v>2421</v>
+        <v>522</v>
       </c>
       <c r="C76">
-        <v>15879.159547835556</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
@@ -1274,10 +1277,10 @@
         <v>3</v>
       </c>
       <c r="B77">
-        <v>2362</v>
+        <v>571</v>
       </c>
       <c r="C77">
-        <v>16506.601026070115</v>
+        <v>187637.4328386733</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -1285,10 +1288,10 @@
         <v>3</v>
       </c>
       <c r="B78">
-        <v>2069</v>
+        <v>580</v>
       </c>
       <c r="C78">
-        <v>18135.339137680952</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -1296,10 +1299,10 @@
         <v>3</v>
       </c>
       <c r="B79">
-        <v>951</v>
+        <v>595</v>
       </c>
       <c r="C79">
-        <v>17568.239596487612</v>
+        <v>131364.08405306729</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -1307,10 +1310,10 @@
         <v>3</v>
       </c>
       <c r="B80">
-        <v>1278</v>
+        <v>634</v>
       </c>
       <c r="C80">
-        <v>18036.96932021953</v>
+        <v>128067.23541614575</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -1318,10 +1321,10 @@
         <v>3</v>
       </c>
       <c r="B81">
-        <v>781</v>
+        <v>703</v>
       </c>
       <c r="C81">
-        <v>18719.671652784327</v>
+        <v>61795.168259892249</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -1340,10 +1343,10 @@
         <v>3</v>
       </c>
       <c r="B83">
-        <v>1501</v>
+        <v>768</v>
       </c>
       <c r="C83">
-        <v>20530.535614897737</v>
+        <v>33148.459440685328</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
@@ -1351,10 +1354,10 @@
         <v>3</v>
       </c>
       <c r="B84">
-        <v>2452</v>
+        <v>772</v>
       </c>
       <c r="C84">
-        <v>21422.849752573147</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
@@ -1362,10 +1365,10 @@
         <v>3</v>
       </c>
       <c r="B85">
-        <v>1374</v>
+        <v>781</v>
       </c>
       <c r="C85">
-        <v>21903.853387666812</v>
+        <v>34588.291215202902</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -1373,10 +1376,10 @@
         <v>3</v>
       </c>
       <c r="B86">
-        <v>2081</v>
+        <v>783</v>
       </c>
       <c r="C86">
-        <v>25507.331305280153</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
@@ -1384,10 +1387,10 @@
         <v>3</v>
       </c>
       <c r="B87">
-        <v>1340</v>
+        <v>802</v>
       </c>
       <c r="C87">
-        <v>27291.339485056553</v>
+        <v>21278.950829061108</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
@@ -1395,10 +1398,10 @@
         <v>3</v>
       </c>
       <c r="B88">
-        <v>1020</v>
+        <v>816</v>
       </c>
       <c r="C88">
-        <v>27640.512465673699</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
@@ -1406,10 +1409,10 @@
         <v>3</v>
       </c>
       <c r="B89">
-        <v>522</v>
+        <v>890</v>
       </c>
       <c r="C89">
-        <v>28375.583495556846</v>
+        <v>246350.12538334605</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
@@ -1417,10 +1420,10 @@
         <v>3</v>
       </c>
       <c r="B90">
-        <v>2442</v>
+        <v>951</v>
       </c>
       <c r="C90">
-        <v>31681.436033528022</v>
+        <v>30501.112008936449</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
@@ -1428,10 +1431,10 @@
         <v>3</v>
       </c>
       <c r="B91">
-        <v>1327</v>
+        <v>1007</v>
       </c>
       <c r="C91">
-        <v>31838.990672440574</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -1439,10 +1442,10 @@
         <v>3</v>
       </c>
       <c r="B92">
-        <v>2431</v>
+        <v>1020</v>
       </c>
       <c r="C92">
-        <v>35644.191992833061</v>
+        <v>22519.81589242462</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
@@ -1450,10 +1453,10 @@
         <v>3</v>
       </c>
       <c r="B93">
-        <v>768</v>
+        <v>1277</v>
       </c>
       <c r="C93">
-        <v>35659.439215953644</v>
+        <v>60220.153089080806</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
@@ -1461,10 +1464,10 @@
         <v>3</v>
       </c>
       <c r="B94">
-        <v>1344</v>
+        <v>1278</v>
       </c>
       <c r="C94">
-        <v>35963.976751075228</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
@@ -1472,10 +1475,10 @@
         <v>3</v>
       </c>
       <c r="B95">
-        <v>104</v>
+        <v>1298</v>
       </c>
       <c r="C95">
-        <v>38496.417494884641</v>
+        <v>301401.93256037129</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
@@ -1505,10 +1508,10 @@
         <v>3</v>
       </c>
       <c r="B98">
-        <v>438</v>
+        <v>1324</v>
       </c>
       <c r="C98">
-        <v>40251.416831324022</v>
+        <v>74196.746858394137</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
@@ -1516,10 +1519,10 @@
         <v>3</v>
       </c>
       <c r="B99">
-        <v>634</v>
+        <v>1327</v>
       </c>
       <c r="C99">
-        <v>41057.668271770664</v>
+        <v>31838.990672440574</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
@@ -1527,10 +1530,10 @@
         <v>3</v>
       </c>
       <c r="B100">
-        <v>2190</v>
+        <v>1340</v>
       </c>
       <c r="C100">
-        <v>41118.888587370981</v>
+        <v>35533.350527718183</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
@@ -1538,10 +1541,10 @@
         <v>3</v>
       </c>
       <c r="B101">
-        <v>1007</v>
+        <v>1344</v>
       </c>
       <c r="C101">
-        <v>42696.597892561709</v>
+        <v>37146.833211802776</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
@@ -1549,10 +1552,10 @@
         <v>3</v>
       </c>
       <c r="B102">
-        <v>452</v>
+        <v>1372</v>
       </c>
       <c r="C102">
-        <v>43799.489265839533</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
@@ -1560,10 +1563,10 @@
         <v>3</v>
       </c>
       <c r="B103">
-        <v>816</v>
+        <v>1374</v>
       </c>
       <c r="C103">
-        <v>47447.576489707164</v>
+        <v>47197.530912325041</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
@@ -1571,10 +1574,10 @@
         <v>3</v>
       </c>
       <c r="B104">
-        <v>2449</v>
+        <v>1380</v>
       </c>
       <c r="C104">
-        <v>47718.488454063969</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
@@ -1582,10 +1585,10 @@
         <v>3</v>
       </c>
       <c r="B105">
-        <v>351</v>
+        <v>1381</v>
       </c>
       <c r="C105">
-        <v>51354.934229929924</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
@@ -1593,10 +1596,10 @@
         <v>3</v>
       </c>
       <c r="B106">
-        <v>1869</v>
+        <v>1384</v>
       </c>
       <c r="C106">
-        <v>52044.632055219103</v>
+        <v>101840.59087657375</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
@@ -1615,10 +1618,10 @@
         <v>3</v>
       </c>
       <c r="B108">
-        <v>2124</v>
+        <v>1501</v>
       </c>
       <c r="C108">
-        <v>52791.487921087763</v>
+        <v>24021.154951741097</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
@@ -1626,10 +1629,10 @@
         <v>3</v>
       </c>
       <c r="B109">
-        <v>2363</v>
+        <v>1518</v>
       </c>
       <c r="C109">
-        <v>54127.538085751112</v>
+        <v>78691.451884710725</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
@@ -1637,10 +1640,10 @@
         <v>3</v>
       </c>
       <c r="B110">
-        <v>595</v>
+        <v>1658</v>
       </c>
       <c r="C110">
-        <v>54174.197632604082</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
@@ -1659,10 +1662,10 @@
         <v>3</v>
       </c>
       <c r="B112">
-        <v>2178</v>
+        <v>1869</v>
       </c>
       <c r="C112">
-        <v>56975.736944821219</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
@@ -1670,10 +1673,10 @@
         <v>3</v>
       </c>
       <c r="B113">
-        <v>2599</v>
+        <v>1996</v>
       </c>
       <c r="C113">
-        <v>59531.16998128454</v>
+        <v>101610.63152690833</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
@@ -1681,10 +1684,10 @@
         <v>3</v>
       </c>
       <c r="B114">
-        <v>1518</v>
+        <v>2069</v>
       </c>
       <c r="C114">
-        <v>63471.353285695448</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.3">
@@ -1692,10 +1695,10 @@
         <v>3</v>
       </c>
       <c r="B115">
-        <v>1372</v>
+        <v>2081</v>
       </c>
       <c r="C115">
-        <v>64553.932829923884</v>
+        <v>35540.327826948735</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.3">
@@ -1714,10 +1717,10 @@
         <v>3</v>
       </c>
       <c r="B117">
-        <v>1277</v>
+        <v>2124</v>
       </c>
       <c r="C117">
-        <v>68540.207905929987</v>
+        <v>87626.868415228644</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
@@ -1725,10 +1728,10 @@
         <v>3</v>
       </c>
       <c r="B118">
-        <v>1996</v>
+        <v>2133</v>
       </c>
       <c r="C118">
-        <v>70326.832086401453</v>
+        <v>126100.59348075089</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
@@ -1736,10 +1739,10 @@
         <v>3</v>
       </c>
       <c r="B119">
-        <v>1324</v>
+        <v>2178</v>
       </c>
       <c r="C119">
-        <v>73489.900387948699</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
@@ -1747,10 +1750,10 @@
         <v>3</v>
       </c>
       <c r="B120">
-        <v>571</v>
+        <v>2190</v>
       </c>
       <c r="C120">
-        <v>79685.515598615108</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
@@ -1769,10 +1772,10 @@
         <v>3</v>
       </c>
       <c r="B122">
-        <v>1381</v>
+        <v>2362</v>
       </c>
       <c r="C122">
-        <v>82010.988601622405</v>
+        <v>18952.135218753476</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
@@ -1780,10 +1783,10 @@
         <v>3</v>
       </c>
       <c r="B123">
-        <v>1384</v>
+        <v>2363</v>
       </c>
       <c r="C123">
-        <v>86910.981482602074</v>
+        <v>38563.286533942613</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
@@ -1802,10 +1805,10 @@
         <v>3</v>
       </c>
       <c r="B125">
-        <v>132</v>
+        <v>2421</v>
       </c>
       <c r="C125">
-        <v>89315.541804343215</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
@@ -1813,10 +1816,10 @@
         <v>3</v>
       </c>
       <c r="B126">
-        <v>703</v>
+        <v>2431</v>
       </c>
       <c r="C126">
-        <v>91911.608434967275</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
@@ -1824,10 +1827,10 @@
         <v>3</v>
       </c>
       <c r="B127">
-        <v>415</v>
+        <v>2433</v>
       </c>
       <c r="C127">
-        <v>101482.12867016949</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
@@ -1835,10 +1838,10 @@
         <v>3</v>
       </c>
       <c r="B128">
-        <v>772</v>
+        <v>2440</v>
       </c>
       <c r="C128">
-        <v>102368.31837304481</v>
+        <v>24757.838493192598</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.3">
@@ -1846,10 +1849,10 @@
         <v>3</v>
       </c>
       <c r="B129">
-        <v>33</v>
+        <v>2442</v>
       </c>
       <c r="C129">
-        <v>111814.41823237992</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.3">
@@ -1857,10 +1860,10 @@
         <v>3</v>
       </c>
       <c r="B130">
-        <v>2133</v>
+        <v>2448</v>
       </c>
       <c r="C130">
-        <v>150059.75520083244</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.3">
@@ -1868,10 +1871,10 @@
         <v>3</v>
       </c>
       <c r="B131">
-        <v>14</v>
+        <v>2449</v>
       </c>
       <c r="C131">
-        <v>159233.28711920604</v>
+        <v>35587.084731704228</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.3">
@@ -1879,10 +1882,10 @@
         <v>3</v>
       </c>
       <c r="B132">
-        <v>20</v>
+        <v>2452</v>
       </c>
       <c r="C132">
-        <v>163831.86029343944</v>
+        <v>17235.15119262048</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.3">
@@ -1901,10 +1904,10 @@
         <v>3</v>
       </c>
       <c r="B134">
-        <v>890</v>
+        <v>2588</v>
       </c>
       <c r="C134">
-        <v>168393.04563881757</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.3">
@@ -1912,10 +1915,10 @@
         <v>3</v>
       </c>
       <c r="B135">
-        <v>1298</v>
+        <v>2599</v>
       </c>
       <c r="C135">
-        <v>387222.13789369148</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.3">
@@ -4101,10 +4104,10 @@
         <v>4</v>
       </c>
       <c r="B334">
-        <v>1045</v>
+        <v>358</v>
       </c>
       <c r="C334">
-        <v>15000</v>
+        <v>77156.847182285579</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.3">
@@ -4112,10 +4115,10 @@
         <v>4</v>
       </c>
       <c r="B335">
-        <v>2366</v>
+        <v>360</v>
       </c>
       <c r="C335">
-        <v>15000</v>
+        <v>141470.97</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.3">
@@ -4123,10 +4126,10 @@
         <v>4</v>
       </c>
       <c r="B336">
-        <v>2799</v>
+        <v>363</v>
       </c>
       <c r="C336">
-        <v>15000</v>
+        <v>76564.066916899654</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.3">
@@ -4145,10 +4148,10 @@
         <v>4</v>
       </c>
       <c r="B338">
-        <v>1823</v>
+        <v>429</v>
       </c>
       <c r="C338">
-        <v>15000</v>
+        <v>47099.4</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.3">
@@ -4156,10 +4159,10 @@
         <v>4</v>
       </c>
       <c r="B339">
-        <v>2330</v>
+        <v>535</v>
       </c>
       <c r="C339">
-        <v>15000</v>
+        <v>72475.414579673743</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.3">
@@ -4189,10 +4192,10 @@
         <v>4</v>
       </c>
       <c r="B342">
-        <v>2755</v>
+        <v>636</v>
       </c>
       <c r="C342">
-        <v>15000</v>
+        <v>40218.51</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.3">
@@ -4200,10 +4203,10 @@
         <v>4</v>
       </c>
       <c r="B343">
-        <v>2692</v>
+        <v>675</v>
       </c>
       <c r="C343">
-        <v>15000</v>
+        <v>33447.636574796554</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.3">
@@ -4225,7 +4228,7 @@
         <v>945</v>
       </c>
       <c r="C345">
-        <v>30703.39941736024</v>
+        <v>34453.4</v>
       </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.3">
@@ -4233,7 +4236,7 @@
         <v>4</v>
       </c>
       <c r="B346">
-        <v>2678</v>
+        <v>1045</v>
       </c>
       <c r="C346">
         <v>15000</v>
@@ -4255,10 +4258,10 @@
         <v>4</v>
       </c>
       <c r="B348">
-        <v>2576</v>
+        <v>1137</v>
       </c>
       <c r="C348">
-        <v>15000</v>
+        <v>196060.36</v>
       </c>
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.3">
@@ -4277,10 +4280,10 @@
         <v>4</v>
       </c>
       <c r="B350">
-        <v>2530</v>
+        <v>1293</v>
       </c>
       <c r="C350">
-        <v>15000</v>
+        <v>100272.94</v>
       </c>
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.3">
@@ -4288,10 +4291,10 @@
         <v>4</v>
       </c>
       <c r="B351">
-        <v>2571</v>
+        <v>1308</v>
       </c>
       <c r="C351">
-        <v>15000</v>
+        <v>33712.998706487044</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.3">
@@ -4310,10 +4313,10 @@
         <v>4</v>
       </c>
       <c r="B353">
-        <v>2691</v>
+        <v>1653</v>
       </c>
       <c r="C353">
-        <v>15000</v>
+        <v>77383.811874679785</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.3">
@@ -4321,7 +4324,7 @@
         <v>4</v>
       </c>
       <c r="B354">
-        <v>2507</v>
+        <v>1823</v>
       </c>
       <c r="C354">
         <v>15000</v>
@@ -4332,10 +4335,10 @@
         <v>4</v>
       </c>
       <c r="B355">
-        <v>2109</v>
+        <v>1906</v>
       </c>
       <c r="C355">
-        <v>15000</v>
+        <v>21140.587231043661</v>
       </c>
     </row>
     <row r="356" spans="1:3" x14ac:dyDescent="0.3">
@@ -4343,10 +4346,10 @@
         <v>4</v>
       </c>
       <c r="B356">
-        <v>2491</v>
+        <v>2015</v>
       </c>
       <c r="C356">
-        <v>15708.103307654304</v>
+        <v>58214.98162022305</v>
       </c>
     </row>
     <row r="357" spans="1:3" x14ac:dyDescent="0.3">
@@ -4354,10 +4357,10 @@
         <v>4</v>
       </c>
       <c r="B357">
-        <v>2680</v>
+        <v>2107</v>
       </c>
       <c r="C357">
-        <v>17653.191516466668</v>
+        <v>109621.02424363823</v>
       </c>
     </row>
     <row r="358" spans="1:3" x14ac:dyDescent="0.3">
@@ -4365,10 +4368,10 @@
         <v>4</v>
       </c>
       <c r="B358">
-        <v>2681</v>
+        <v>2109</v>
       </c>
       <c r="C358">
-        <v>18087.411572689049</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.3">
@@ -4387,10 +4390,10 @@
         <v>4</v>
       </c>
       <c r="B360">
-        <v>2359</v>
+        <v>2118</v>
       </c>
       <c r="C360">
-        <v>17115.396352551164</v>
+        <v>69687.832795976705</v>
       </c>
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.3">
@@ -4409,10 +4412,10 @@
         <v>4</v>
       </c>
       <c r="B362">
-        <v>1906</v>
+        <v>2211</v>
       </c>
       <c r="C362">
-        <v>21140.587231043661</v>
+        <v>74015.535398273918</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.3">
@@ -4420,10 +4423,10 @@
         <v>4</v>
       </c>
       <c r="B363">
-        <v>2698</v>
+        <v>2308</v>
       </c>
       <c r="C363">
-        <v>21540.450340488205</v>
+        <v>27283.948571802139</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.3">
@@ -4431,10 +4434,10 @@
         <v>4</v>
       </c>
       <c r="B364">
-        <v>2767</v>
+        <v>2330</v>
       </c>
       <c r="C364">
-        <v>21589.803591399374</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.3">
@@ -4442,10 +4445,10 @@
         <v>4</v>
       </c>
       <c r="B365">
-        <v>2383</v>
+        <v>2359</v>
       </c>
       <c r="C365">
-        <v>25236.019576771883</v>
+        <v>17115.396352551164</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.3">
@@ -4453,10 +4456,10 @@
         <v>4</v>
       </c>
       <c r="B366">
-        <v>2697</v>
+        <v>2366</v>
       </c>
       <c r="C366">
-        <v>27058.895143994421</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.3">
@@ -4464,10 +4467,10 @@
         <v>4</v>
       </c>
       <c r="B367">
-        <v>2308</v>
+        <v>2383</v>
       </c>
       <c r="C367">
-        <v>27283.948571802139</v>
+        <v>25236.019576771883</v>
       </c>
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.3">
@@ -4475,10 +4478,10 @@
         <v>4</v>
       </c>
       <c r="B368">
-        <v>2709</v>
+        <v>2491</v>
       </c>
       <c r="C368">
-        <v>29749.635377291357</v>
+        <v>15708.103307654304</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.3">
@@ -4486,10 +4489,10 @@
         <v>4</v>
       </c>
       <c r="B369">
-        <v>675</v>
+        <v>2507</v>
       </c>
       <c r="C369">
-        <v>33447.636574796554</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.3">
@@ -4497,10 +4500,10 @@
         <v>4</v>
       </c>
       <c r="B370">
-        <v>1308</v>
+        <v>2530</v>
       </c>
       <c r="C370">
-        <v>33712.998706487044</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="371" spans="1:3" x14ac:dyDescent="0.3">
@@ -4508,10 +4511,10 @@
         <v>4</v>
       </c>
       <c r="B371">
-        <v>636</v>
+        <v>2571</v>
       </c>
       <c r="C371">
-        <v>36468.506339702646</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="372" spans="1:3" x14ac:dyDescent="0.3">
@@ -4519,10 +4522,10 @@
         <v>4</v>
       </c>
       <c r="B372">
-        <v>429</v>
+        <v>2576</v>
       </c>
       <c r="C372">
-        <v>43349.400638036488</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.3">
@@ -4530,10 +4533,10 @@
         <v>4</v>
       </c>
       <c r="B373">
-        <v>2015</v>
+        <v>2678</v>
       </c>
       <c r="C373">
-        <v>58214.98162022305</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="374" spans="1:3" x14ac:dyDescent="0.3">
@@ -4541,10 +4544,10 @@
         <v>4</v>
       </c>
       <c r="B374">
-        <v>2696</v>
+        <v>2680</v>
       </c>
       <c r="C374">
-        <v>68173.211828627595</v>
+        <v>17653.191516466668</v>
       </c>
     </row>
     <row r="375" spans="1:3" x14ac:dyDescent="0.3">
@@ -4552,10 +4555,10 @@
         <v>4</v>
       </c>
       <c r="B375">
-        <v>2118</v>
+        <v>2681</v>
       </c>
       <c r="C375">
-        <v>69687.832795976705</v>
+        <v>18087.411572689049</v>
       </c>
     </row>
     <row r="376" spans="1:3" x14ac:dyDescent="0.3">
@@ -4563,10 +4566,10 @@
         <v>4</v>
       </c>
       <c r="B376">
-        <v>535</v>
+        <v>2691</v>
       </c>
       <c r="C376">
-        <v>72475.414579673743</v>
+        <v>30743.31</v>
       </c>
     </row>
     <row r="377" spans="1:3" x14ac:dyDescent="0.3">
@@ -4574,10 +4577,10 @@
         <v>4</v>
       </c>
       <c r="B377">
-        <v>2211</v>
+        <v>2692</v>
       </c>
       <c r="C377">
-        <v>74015.535398273918</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="378" spans="1:3" x14ac:dyDescent="0.3">
@@ -4585,10 +4588,10 @@
         <v>4</v>
       </c>
       <c r="B378">
-        <v>2768</v>
+        <v>2696</v>
       </c>
       <c r="C378">
-        <v>74786.275879616267</v>
+        <v>68173.211828627595</v>
       </c>
     </row>
     <row r="379" spans="1:3" x14ac:dyDescent="0.3">
@@ -4596,10 +4599,10 @@
         <v>4</v>
       </c>
       <c r="B379">
-        <v>363</v>
+        <v>2697</v>
       </c>
       <c r="C379">
-        <v>76564.066916899654</v>
+        <v>27058.895143994421</v>
       </c>
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.3">
@@ -4607,10 +4610,10 @@
         <v>4</v>
       </c>
       <c r="B380">
-        <v>358</v>
+        <v>2698</v>
       </c>
       <c r="C380">
-        <v>77156.847182285579</v>
+        <v>21540.450340488205</v>
       </c>
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.3">
@@ -4618,10 +4621,10 @@
         <v>4</v>
       </c>
       <c r="B381">
-        <v>1653</v>
+        <v>2709</v>
       </c>
       <c r="C381">
-        <v>77383.811874679785</v>
+        <v>29749.635377291357</v>
       </c>
     </row>
     <row r="382" spans="1:3" x14ac:dyDescent="0.3">
@@ -4640,10 +4643,10 @@
         <v>4</v>
       </c>
       <c r="B383">
-        <v>1293</v>
+        <v>2755</v>
       </c>
       <c r="C383">
-        <v>96522.93633956174</v>
+        <v>15204.97</v>
       </c>
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.3">
@@ -4651,10 +4654,10 @@
         <v>4</v>
       </c>
       <c r="B384">
-        <v>2107</v>
+        <v>2767</v>
       </c>
       <c r="C384">
-        <v>109621.02424363823</v>
+        <v>21589.803591399374</v>
       </c>
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.3">
@@ -4662,10 +4665,10 @@
         <v>4</v>
       </c>
       <c r="B385">
-        <v>360</v>
+        <v>2768</v>
       </c>
       <c r="C385">
-        <v>126470.96829860304</v>
+        <v>74786.275879616267</v>
       </c>
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.3">
@@ -4673,10 +4676,10 @@
         <v>4</v>
       </c>
       <c r="B386">
-        <v>1137</v>
+        <v>2799</v>
       </c>
       <c r="C386">
-        <v>196060.35945056166</v>
+        <v>15000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajuste meta filial 3
</commit_message>
<xml_diff>
--- a/data/meta_rca.xlsx
+++ b/data/meta_rca.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61834950-D982-4808-82C2-6CB789668F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9DFBEE-AE15-4FDC-80A5-B0A2BE5ADEAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{91476B03-704D-4E23-9E63-F1D303A50E23}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$C$370</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$C$371</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -428,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{412D1898-A7F6-4EAA-ABB1-3B7D2190621B}">
-  <dimension ref="A1:C370"/>
+  <dimension ref="A1:C371"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
@@ -1412,7 +1412,7 @@
         <v>2363</v>
       </c>
       <c r="C89">
-        <v>38563.286533942613</v>
+        <v>37749.035579222575</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
@@ -1423,7 +1423,7 @@
         <v>2124</v>
       </c>
       <c r="C90">
-        <v>87626.868415228644</v>
+        <v>85776.656265820027</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
@@ -1434,7 +1434,7 @@
         <v>1020</v>
       </c>
       <c r="C91">
-        <v>22519.81589242462</v>
+        <v>22044.317478294732</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -1445,7 +1445,7 @@
         <v>768</v>
       </c>
       <c r="C92">
-        <v>33148.459440685328</v>
+        <v>32448.540757060699</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
@@ -1456,7 +1456,7 @@
         <v>781</v>
       </c>
       <c r="C93">
-        <v>34588.291215202902</v>
+        <v>33857.970963081119</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
@@ -1467,7 +1467,7 @@
         <v>951</v>
       </c>
       <c r="C94">
-        <v>30501.112008936449</v>
+        <v>29857.091184844103</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
@@ -1478,7 +1478,7 @@
         <v>2362</v>
       </c>
       <c r="C95">
-        <v>18952.135218753476</v>
+        <v>18551.967194115055</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
@@ -1489,7 +1489,7 @@
         <v>1340</v>
       </c>
       <c r="C96">
-        <v>35533.350527718183</v>
+        <v>34783.075662889692</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
@@ -1500,7 +1500,7 @@
         <v>1324</v>
       </c>
       <c r="C97">
-        <v>74196.746858394137</v>
+        <v>72630.107253821217</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
@@ -1511,7 +1511,7 @@
         <v>1344</v>
       </c>
       <c r="C98">
-        <v>37146.833211802776</v>
+        <v>36362.490197342289</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
@@ -1522,7 +1522,7 @@
         <v>802</v>
       </c>
       <c r="C99">
-        <v>21278.950829061108</v>
+        <v>20829.652867572444</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
@@ -1533,7 +1533,7 @@
         <v>2452</v>
       </c>
       <c r="C100">
-        <v>17235.15119262048</v>
+        <v>16871.236713988499</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
@@ -1544,7 +1544,7 @@
         <v>703</v>
       </c>
       <c r="C101">
-        <v>61795.168259892249</v>
+        <v>60490.383858064502</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
@@ -1555,7 +1555,7 @@
         <v>2449</v>
       </c>
       <c r="C102">
-        <v>35587.084731704228</v>
+        <v>34835.675287050486</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
@@ -1566,7 +1566,7 @@
         <v>1277</v>
       </c>
       <c r="C103">
-        <v>60220.153089080806</v>
+        <v>58948.624608150851</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
@@ -1577,7 +1577,7 @@
         <v>14</v>
       </c>
       <c r="C104">
-        <v>114589.7365638465</v>
+        <v>110975.932431325</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
@@ -1588,7 +1588,7 @@
         <v>2081</v>
       </c>
       <c r="C105">
-        <v>35540.327826948735</v>
+        <v>34789.905638770229</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
@@ -1599,7 +1599,7 @@
         <v>1501</v>
       </c>
       <c r="C106">
-        <v>24021.154951741097</v>
+        <v>23513.956263275646</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
@@ -1610,7 +1610,7 @@
         <v>1374</v>
       </c>
       <c r="C107">
-        <v>47197.530912325041</v>
+        <v>46200.970762505778</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
@@ -1621,7 +1621,7 @@
         <v>2440</v>
       </c>
       <c r="C108">
-        <v>24757.838493192598</v>
+        <v>25112.645889198313</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
@@ -1758,13 +1758,13 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B121">
-        <v>326</v>
+        <v>2448</v>
       </c>
       <c r="C121">
-        <v>11583.888071768148</v>
+        <v>18369.760315498828</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
@@ -1772,10 +1772,10 @@
         <v>7</v>
       </c>
       <c r="B122">
-        <v>716</v>
+        <v>326</v>
       </c>
       <c r="C122">
-        <v>42273.283164882057</v>
+        <v>11583.888071768148</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
@@ -1783,10 +1783,10 @@
         <v>7</v>
       </c>
       <c r="B123">
-        <v>749</v>
+        <v>716</v>
       </c>
       <c r="C123">
-        <v>10505.487010089315</v>
+        <v>42273.283164882057</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
@@ -1794,10 +1794,10 @@
         <v>7</v>
       </c>
       <c r="B124">
-        <v>766</v>
+        <v>749</v>
       </c>
       <c r="C124">
-        <v>2721.2911093308385</v>
+        <v>10505.487010089315</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
@@ -1805,10 +1805,10 @@
         <v>7</v>
       </c>
       <c r="B125">
-        <v>793</v>
+        <v>766</v>
       </c>
       <c r="C125">
-        <v>4045.8700792817908</v>
+        <v>2721.2911093308385</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
@@ -1816,10 +1816,10 @@
         <v>7</v>
       </c>
       <c r="B126">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="C126">
-        <v>3097.9601604174809</v>
+        <v>4045.8700792817908</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
@@ -1827,10 +1827,10 @@
         <v>7</v>
       </c>
       <c r="B127">
-        <v>2653</v>
+        <v>794</v>
       </c>
       <c r="C127">
-        <v>15000</v>
+        <v>3097.9601604174809</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
@@ -1838,7 +1838,7 @@
         <v>7</v>
       </c>
       <c r="B128">
-        <v>2566</v>
+        <v>2653</v>
       </c>
       <c r="C128">
         <v>15000</v>
@@ -1849,10 +1849,10 @@
         <v>7</v>
       </c>
       <c r="B129">
-        <v>933</v>
+        <v>2566</v>
       </c>
       <c r="C129">
-        <v>297.19589624545239</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.3">
@@ -1860,10 +1860,10 @@
         <v>7</v>
       </c>
       <c r="B130">
-        <v>2804</v>
+        <v>933</v>
       </c>
       <c r="C130">
-        <v>15000</v>
+        <v>297.19589624545239</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.3">
@@ -1871,10 +1871,10 @@
         <v>7</v>
       </c>
       <c r="B131">
-        <v>966</v>
+        <v>2804</v>
       </c>
       <c r="C131">
-        <v>470.04180850358654</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.3">
@@ -1882,10 +1882,10 @@
         <v>7</v>
       </c>
       <c r="B132">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="C132">
-        <v>8441.7316040323221</v>
+        <v>470.04180850358654</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.3">
@@ -1893,10 +1893,10 @@
         <v>7</v>
       </c>
       <c r="B133">
-        <v>2797</v>
+        <v>970</v>
       </c>
       <c r="C133">
-        <v>15000</v>
+        <v>8441.7316040323221</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.3">
@@ -1904,7 +1904,7 @@
         <v>7</v>
       </c>
       <c r="B134">
-        <v>2750</v>
+        <v>2797</v>
       </c>
       <c r="C134">
         <v>15000</v>
@@ -1915,10 +1915,10 @@
         <v>7</v>
       </c>
       <c r="B135">
-        <v>1486</v>
+        <v>2750</v>
       </c>
       <c r="C135">
-        <v>1539.4432021025718</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.3">
@@ -1926,10 +1926,10 @@
         <v>7</v>
       </c>
       <c r="B136">
-        <v>2744</v>
+        <v>1486</v>
       </c>
       <c r="C136">
-        <v>15000</v>
+        <v>1539.4432021025718</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.3">
@@ -1937,7 +1937,7 @@
         <v>7</v>
       </c>
       <c r="B137">
-        <v>2748</v>
+        <v>2744</v>
       </c>
       <c r="C137">
         <v>15000</v>
@@ -1948,7 +1948,7 @@
         <v>7</v>
       </c>
       <c r="B138">
-        <v>2798</v>
+        <v>2748</v>
       </c>
       <c r="C138">
         <v>15000</v>
@@ -1959,7 +1959,7 @@
         <v>7</v>
       </c>
       <c r="B139">
-        <v>2673</v>
+        <v>2798</v>
       </c>
       <c r="C139">
         <v>15000</v>
@@ -1970,7 +1970,7 @@
         <v>7</v>
       </c>
       <c r="B140">
-        <v>1492</v>
+        <v>2673</v>
       </c>
       <c r="C140">
         <v>15000</v>
@@ -1981,7 +1981,7 @@
         <v>7</v>
       </c>
       <c r="B141">
-        <v>2659</v>
+        <v>1492</v>
       </c>
       <c r="C141">
         <v>15000</v>
@@ -1992,10 +1992,10 @@
         <v>7</v>
       </c>
       <c r="B142">
-        <v>1881</v>
+        <v>2659</v>
       </c>
       <c r="C142">
-        <v>0</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.3">
@@ -2003,10 +2003,10 @@
         <v>7</v>
       </c>
       <c r="B143">
-        <v>2090</v>
+        <v>1881</v>
       </c>
       <c r="C143">
-        <v>364.12661068264646</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.3">
@@ -2014,10 +2014,10 @@
         <v>7</v>
       </c>
       <c r="B144">
-        <v>2718</v>
+        <v>2090</v>
       </c>
       <c r="C144">
-        <v>15000</v>
+        <v>364.12661068264646</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
@@ -2025,7 +2025,7 @@
         <v>7</v>
       </c>
       <c r="B145">
-        <v>2621</v>
+        <v>2718</v>
       </c>
       <c r="C145">
         <v>15000</v>
@@ -2036,7 +2036,7 @@
         <v>7</v>
       </c>
       <c r="B146">
-        <v>2131</v>
+        <v>2621</v>
       </c>
       <c r="C146">
         <v>15000</v>
@@ -2047,7 +2047,7 @@
         <v>7</v>
       </c>
       <c r="B147">
-        <v>2758</v>
+        <v>2131</v>
       </c>
       <c r="C147">
         <v>15000</v>
@@ -2058,7 +2058,7 @@
         <v>7</v>
       </c>
       <c r="B148">
-        <v>2803</v>
+        <v>2758</v>
       </c>
       <c r="C148">
         <v>15000</v>
@@ -2069,10 +2069,10 @@
         <v>7</v>
       </c>
       <c r="B149">
-        <v>2323</v>
+        <v>2803</v>
       </c>
       <c r="C149">
-        <v>4315.5834415491463</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.3">
@@ -2080,10 +2080,10 @@
         <v>7</v>
       </c>
       <c r="B150">
-        <v>952</v>
+        <v>2323</v>
       </c>
       <c r="C150">
-        <v>15000</v>
+        <v>4315.5834415491463</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.3">
@@ -2091,7 +2091,7 @@
         <v>7</v>
       </c>
       <c r="B151">
-        <v>2795</v>
+        <v>952</v>
       </c>
       <c r="C151">
         <v>15000</v>
@@ -2102,7 +2102,7 @@
         <v>7</v>
       </c>
       <c r="B152">
-        <v>2722</v>
+        <v>2795</v>
       </c>
       <c r="C152">
         <v>15000</v>
@@ -2113,7 +2113,7 @@
         <v>7</v>
       </c>
       <c r="B153">
-        <v>2729</v>
+        <v>2722</v>
       </c>
       <c r="C153">
         <v>15000</v>
@@ -2124,7 +2124,7 @@
         <v>7</v>
       </c>
       <c r="B154">
-        <v>2735</v>
+        <v>2729</v>
       </c>
       <c r="C154">
         <v>15000</v>
@@ -2135,7 +2135,7 @@
         <v>7</v>
       </c>
       <c r="B155">
-        <v>2747</v>
+        <v>2735</v>
       </c>
       <c r="C155">
         <v>15000</v>
@@ -2146,10 +2146,10 @@
         <v>7</v>
       </c>
       <c r="B156">
-        <v>2583</v>
+        <v>2747</v>
       </c>
       <c r="C156">
-        <v>372.78982921236781</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.3">
@@ -2157,10 +2157,10 @@
         <v>7</v>
       </c>
       <c r="B157">
-        <v>2796</v>
+        <v>2583</v>
       </c>
       <c r="C157">
-        <v>15000</v>
+        <v>372.78982921236781</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.3">
@@ -2168,10 +2168,10 @@
         <v>7</v>
       </c>
       <c r="B158">
-        <v>2794</v>
+        <v>2796</v>
       </c>
       <c r="C158">
-        <v>15734.429283546768</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.3">
@@ -2179,10 +2179,10 @@
         <v>7</v>
       </c>
       <c r="B159">
-        <v>2629</v>
+        <v>2794</v>
       </c>
       <c r="C159">
-        <v>1395.0502829908833</v>
+        <v>15734.429283546768</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.3">
@@ -2190,10 +2190,10 @@
         <v>7</v>
       </c>
       <c r="B160">
-        <v>2753</v>
+        <v>2629</v>
       </c>
       <c r="C160">
-        <v>15904.153722809857</v>
+        <v>1395.0502829908833</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.3">
@@ -2201,10 +2201,10 @@
         <v>7</v>
       </c>
       <c r="B161">
-        <v>2772</v>
+        <v>2753</v>
       </c>
       <c r="C161">
-        <v>14597.852354115106</v>
+        <v>15904.153722809857</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.3">
@@ -2212,10 +2212,10 @@
         <v>7</v>
       </c>
       <c r="B162">
-        <v>2786</v>
+        <v>2772</v>
       </c>
       <c r="C162">
-        <v>17447.146475612244</v>
+        <v>14597.852354115106</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.3">
@@ -2223,10 +2223,10 @@
         <v>7</v>
       </c>
       <c r="B163">
-        <v>2742</v>
+        <v>2786</v>
       </c>
       <c r="C163">
-        <v>18302.407456884546</v>
+        <v>17447.146475612244</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.3">
@@ -2234,10 +2234,10 @@
         <v>7</v>
       </c>
       <c r="B164">
-        <v>2765</v>
+        <v>2742</v>
       </c>
       <c r="C164">
-        <v>18473.070599983104</v>
+        <v>18302.407456884546</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.3">
@@ -2245,10 +2245,10 @@
         <v>7</v>
       </c>
       <c r="B165">
-        <v>2783</v>
+        <v>2765</v>
       </c>
       <c r="C165">
-        <v>18491.42621835613</v>
+        <v>18473.070599983104</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.3">
@@ -2256,10 +2256,10 @@
         <v>7</v>
       </c>
       <c r="B166">
-        <v>2163</v>
+        <v>2783</v>
       </c>
       <c r="C166">
-        <v>20188.817639150911</v>
+        <v>18491.42621835613</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.3">
@@ -2267,10 +2267,10 @@
         <v>7</v>
       </c>
       <c r="B167">
-        <v>2745</v>
+        <v>2163</v>
       </c>
       <c r="C167">
-        <v>21573.066503658221</v>
+        <v>20188.817639150911</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.3">
@@ -2278,10 +2278,10 @@
         <v>7</v>
       </c>
       <c r="B168">
-        <v>2496</v>
+        <v>2745</v>
       </c>
       <c r="C168">
-        <v>21936.850110828418</v>
+        <v>21573.066503658221</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.3">
@@ -2289,10 +2289,10 @@
         <v>7</v>
       </c>
       <c r="B169">
-        <v>2544</v>
+        <v>2496</v>
       </c>
       <c r="C169">
-        <v>22948.656914405998</v>
+        <v>21936.850110828418</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.3">
@@ -2300,10 +2300,10 @@
         <v>7</v>
       </c>
       <c r="B170">
-        <v>2655</v>
+        <v>2544</v>
       </c>
       <c r="C170">
-        <v>22969.835191461934</v>
+        <v>22948.656914405998</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.3">
@@ -2311,10 +2311,10 @@
         <v>7</v>
       </c>
       <c r="B171">
-        <v>2346</v>
+        <v>2655</v>
       </c>
       <c r="C171">
-        <v>23899.815722304877</v>
+        <v>22969.835191461934</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.3">
@@ -2322,10 +2322,10 @@
         <v>7</v>
       </c>
       <c r="B172">
-        <v>2757</v>
+        <v>2346</v>
       </c>
       <c r="C172">
-        <v>24367.63554870987</v>
+        <v>23899.815722304877</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.3">
@@ -2333,10 +2333,10 @@
         <v>7</v>
       </c>
       <c r="B173">
-        <v>2258</v>
+        <v>2757</v>
       </c>
       <c r="C173">
-        <v>25383.729414965957</v>
+        <v>24367.63554870987</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.3">
@@ -2344,10 +2344,10 @@
         <v>7</v>
       </c>
       <c r="B174">
-        <v>1642</v>
+        <v>2258</v>
       </c>
       <c r="C174">
-        <v>25961.269431081178</v>
+        <v>25383.729414965957</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.3">
@@ -2355,10 +2355,10 @@
         <v>7</v>
       </c>
       <c r="B175">
-        <v>2601</v>
+        <v>1642</v>
       </c>
       <c r="C175">
-        <v>26114.806101394686</v>
+        <v>25961.269431081178</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.3">
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="B176">
-        <v>2266</v>
+        <v>2601</v>
       </c>
       <c r="C176">
-        <v>26758.340224927189</v>
+        <v>26114.806101394686</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.3">
@@ -2377,10 +2377,10 @@
         <v>7</v>
       </c>
       <c r="B177">
-        <v>2737</v>
+        <v>2266</v>
       </c>
       <c r="C177">
-        <v>28244.581688216211</v>
+        <v>26758.340224927189</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.3">
@@ -2388,10 +2388,10 @@
         <v>7</v>
       </c>
       <c r="B178">
-        <v>1499</v>
+        <v>2737</v>
       </c>
       <c r="C178">
-        <v>28490.359800262864</v>
+        <v>28244.581688216211</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.3">
@@ -2399,10 +2399,10 @@
         <v>7</v>
       </c>
       <c r="B179">
-        <v>2671</v>
+        <v>1499</v>
       </c>
       <c r="C179">
-        <v>28546.584200486643</v>
+        <v>28490.359800262864</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.3">
@@ -2410,10 +2410,10 @@
         <v>7</v>
       </c>
       <c r="B180">
-        <v>1259</v>
+        <v>2671</v>
       </c>
       <c r="C180">
-        <v>31615.285240570891</v>
+        <v>28546.584200486643</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.3">
@@ -2421,10 +2421,10 @@
         <v>7</v>
       </c>
       <c r="B181">
-        <v>854</v>
+        <v>1259</v>
       </c>
       <c r="C181">
-        <v>33482.503851376794</v>
+        <v>31615.285240570891</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.3">
@@ -2432,10 +2432,10 @@
         <v>7</v>
       </c>
       <c r="B182">
-        <v>1539</v>
+        <v>854</v>
       </c>
       <c r="C182">
-        <v>35993.084223857455</v>
+        <v>33482.503851376794</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.3">
@@ -2443,10 +2443,10 @@
         <v>7</v>
       </c>
       <c r="B183">
-        <v>2684</v>
+        <v>1539</v>
       </c>
       <c r="C183">
-        <v>45252.345760045195</v>
+        <v>35993.084223857455</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.3">
@@ -2454,10 +2454,10 @@
         <v>7</v>
       </c>
       <c r="B184">
-        <v>2635</v>
+        <v>2684</v>
       </c>
       <c r="C184">
-        <v>52043.121570446521</v>
+        <v>45252.345760045195</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.3">
@@ -2465,10 +2465,10 @@
         <v>7</v>
       </c>
       <c r="B185">
-        <v>2761</v>
+        <v>2635</v>
       </c>
       <c r="C185">
-        <v>202.96360278639503</v>
+        <v>52043.121570446521</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.3">
@@ -2476,10 +2476,10 @@
         <v>7</v>
       </c>
       <c r="B186">
-        <v>2762</v>
+        <v>2761</v>
       </c>
       <c r="C186">
-        <v>198.98259374923848</v>
+        <v>202.96360278639503</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.3">
@@ -2487,10 +2487,10 @@
         <v>7</v>
       </c>
       <c r="B187">
-        <v>2714</v>
+        <v>2762</v>
       </c>
       <c r="C187">
-        <v>55830.373042976338</v>
+        <v>198.98259374923848</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.3">
@@ -2498,10 +2498,10 @@
         <v>7</v>
       </c>
       <c r="B188">
-        <v>1853</v>
+        <v>2714</v>
       </c>
       <c r="C188">
-        <v>56456.262352775535</v>
+        <v>55830.373042976338</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.3">
@@ -2509,10 +2509,10 @@
         <v>7</v>
       </c>
       <c r="B189">
-        <v>2663</v>
+        <v>1853</v>
       </c>
       <c r="C189">
-        <v>58943.069564306577</v>
+        <v>56456.262352775535</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.3">
@@ -2520,10 +2520,10 @@
         <v>7</v>
       </c>
       <c r="B190">
-        <v>2784</v>
+        <v>2663</v>
       </c>
       <c r="C190">
-        <v>6457.513329441299</v>
+        <v>58943.069564306577</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.3">
@@ -2531,10 +2531,10 @@
         <v>7</v>
       </c>
       <c r="B191">
-        <v>2785</v>
+        <v>2784</v>
       </c>
       <c r="C191">
-        <v>289.05292321490498</v>
+        <v>6457.513329441299</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.3">
@@ -2542,10 +2542,10 @@
         <v>7</v>
       </c>
       <c r="B192">
-        <v>2652</v>
+        <v>2785</v>
       </c>
       <c r="C192">
-        <v>59374.941390303684</v>
+        <v>289.05292321490498</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.3">
@@ -2553,10 +2553,10 @@
         <v>7</v>
       </c>
       <c r="B193">
-        <v>2494</v>
+        <v>2652</v>
       </c>
       <c r="C193">
-        <v>63312.687298065466</v>
+        <v>59374.941390303684</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.3">
@@ -2564,10 +2564,10 @@
         <v>7</v>
       </c>
       <c r="B194">
-        <v>1466</v>
+        <v>2494</v>
       </c>
       <c r="C194">
-        <v>83570.304181871368</v>
+        <v>63312.687298065466</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.3">
@@ -2575,10 +2575,10 @@
         <v>7</v>
       </c>
       <c r="B195">
-        <v>2375</v>
+        <v>1466</v>
       </c>
       <c r="C195">
-        <v>95649.283493875162</v>
+        <v>83570.304181871368</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.3">
@@ -2586,10 +2586,10 @@
         <v>7</v>
       </c>
       <c r="B196">
-        <v>2261</v>
+        <v>2375</v>
       </c>
       <c r="C196">
-        <v>96210.597317517779</v>
+        <v>95649.283493875162</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.3">
@@ -2597,10 +2597,10 @@
         <v>7</v>
       </c>
       <c r="B197">
-        <v>2674</v>
+        <v>2261</v>
       </c>
       <c r="C197">
-        <v>148716.29205725499</v>
+        <v>96210.597317517779</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.3">
@@ -2608,10 +2608,10 @@
         <v>7</v>
       </c>
       <c r="B198">
-        <v>1873</v>
+        <v>2674</v>
       </c>
       <c r="C198">
-        <v>232710.61954604008</v>
+        <v>148716.29205725499</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.3">
@@ -2619,10 +2619,10 @@
         <v>7</v>
       </c>
       <c r="B199">
-        <v>818</v>
+        <v>1873</v>
       </c>
       <c r="C199">
-        <v>271482.93511535402</v>
+        <v>232710.61954604008</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.3">
@@ -2630,21 +2630,21 @@
         <v>7</v>
       </c>
       <c r="B200">
-        <v>6564</v>
+        <v>818</v>
       </c>
       <c r="C200">
-        <v>8524.7972112499265</v>
+        <v>271482.93511535402</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B201">
-        <v>326</v>
+        <v>6564</v>
       </c>
       <c r="C201">
-        <v>2164.4492035823141</v>
+        <v>8524.7972112499265</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.3">
@@ -2652,10 +2652,10 @@
         <v>9</v>
       </c>
       <c r="B202">
-        <v>949</v>
+        <v>326</v>
       </c>
       <c r="C202">
-        <v>34697.872761327882</v>
+        <v>2164.4492035823141</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.3">
@@ -2663,10 +2663,10 @@
         <v>9</v>
       </c>
       <c r="B203">
-        <v>2402</v>
+        <v>949</v>
       </c>
       <c r="C203">
-        <v>15000</v>
+        <v>34697.872761327882</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.3">
@@ -2674,10 +2674,10 @@
         <v>9</v>
       </c>
       <c r="B204">
-        <v>2145</v>
+        <v>2402</v>
       </c>
       <c r="C204">
-        <v>15774.041336161203</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.3">
@@ -2685,10 +2685,10 @@
         <v>9</v>
       </c>
       <c r="B205">
-        <v>2082</v>
+        <v>2145</v>
       </c>
       <c r="C205">
-        <v>17020.693875270284</v>
+        <v>15774.041336161203</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.3">
@@ -2696,10 +2696,10 @@
         <v>9</v>
       </c>
       <c r="B206">
-        <v>1585</v>
+        <v>2082</v>
       </c>
       <c r="C206">
-        <v>18166.851997739006</v>
+        <v>17020.693875270284</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.3">
@@ -2707,10 +2707,10 @@
         <v>9</v>
       </c>
       <c r="B207">
-        <v>2492</v>
+        <v>1585</v>
       </c>
       <c r="C207">
-        <v>26837.669420235306</v>
+        <v>18166.851997739006</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.3">
@@ -2718,10 +2718,10 @@
         <v>9</v>
       </c>
       <c r="B208">
-        <v>2567</v>
+        <v>2492</v>
       </c>
       <c r="C208">
-        <v>26971.263423143064</v>
+        <v>26837.669420235306</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.3">
@@ -2729,10 +2729,10 @@
         <v>9</v>
       </c>
       <c r="B209">
-        <v>2223</v>
+        <v>2567</v>
       </c>
       <c r="C209">
-        <v>27298.800416513488</v>
+        <v>26971.263423143064</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.3">
@@ -2740,10 +2740,10 @@
         <v>9</v>
       </c>
       <c r="B210">
-        <v>2392</v>
+        <v>2223</v>
       </c>
       <c r="C210">
-        <v>30676.602249814285</v>
+        <v>27298.800416513488</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.3">
@@ -2751,10 +2751,10 @@
         <v>9</v>
       </c>
       <c r="B211">
-        <v>2325</v>
+        <v>2392</v>
       </c>
       <c r="C211">
-        <v>31156.909970474022</v>
+        <v>30676.602249814285</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.3">
@@ -2762,10 +2762,10 @@
         <v>9</v>
       </c>
       <c r="B212">
-        <v>2568</v>
+        <v>2325</v>
       </c>
       <c r="C212">
-        <v>32092.853522185076</v>
+        <v>31156.909970474022</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.3">
@@ -2773,10 +2773,10 @@
         <v>9</v>
       </c>
       <c r="B213">
-        <v>2183</v>
+        <v>2568</v>
       </c>
       <c r="C213">
-        <v>210614.53897343809</v>
+        <v>32092.853522185076</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.3">
@@ -2784,10 +2784,10 @@
         <v>9</v>
       </c>
       <c r="B214">
-        <v>2333</v>
+        <v>2183</v>
       </c>
       <c r="C214">
-        <v>32617.06341133004</v>
+        <v>210614.53897343809</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.3">
@@ -2795,10 +2795,10 @@
         <v>9</v>
       </c>
       <c r="B215">
-        <v>2606</v>
+        <v>2333</v>
       </c>
       <c r="C215">
-        <v>33628.885491502668</v>
+        <v>32617.06341133004</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.3">
@@ -2806,10 +2806,10 @@
         <v>9</v>
       </c>
       <c r="B216">
-        <v>1834</v>
+        <v>2606</v>
       </c>
       <c r="C216">
-        <v>35459.202393156709</v>
+        <v>33628.885491502668</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.3">
@@ -2817,10 +2817,10 @@
         <v>9</v>
       </c>
       <c r="B217">
-        <v>2647</v>
+        <v>1834</v>
       </c>
       <c r="C217">
-        <v>36315.180244363895</v>
+        <v>35459.202393156709</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.3">
@@ -2828,10 +2828,10 @@
         <v>9</v>
       </c>
       <c r="B218">
-        <v>2411</v>
+        <v>2647</v>
       </c>
       <c r="C218">
-        <v>38320.521466522208</v>
+        <v>36315.180244363895</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.3">
@@ -2839,10 +2839,10 @@
         <v>9</v>
       </c>
       <c r="B219">
-        <v>2394</v>
+        <v>2411</v>
       </c>
       <c r="C219">
-        <v>42875.802194412019</v>
+        <v>38320.521466522208</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.3">
@@ -2850,10 +2850,10 @@
         <v>9</v>
       </c>
       <c r="B220">
-        <v>2341</v>
+        <v>2394</v>
       </c>
       <c r="C220">
-        <v>43645.539701259404</v>
+        <v>42875.802194412019</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.3">
@@ -2861,10 +2861,10 @@
         <v>9</v>
       </c>
       <c r="B221">
-        <v>2613</v>
+        <v>2341</v>
       </c>
       <c r="C221">
-        <v>43792.4702586618</v>
+        <v>43645.539701259404</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.3">
@@ -2872,10 +2872,10 @@
         <v>9</v>
       </c>
       <c r="B222">
-        <v>1456</v>
+        <v>2613</v>
       </c>
       <c r="C222">
-        <v>51425.245286726502</v>
+        <v>43792.4702586618</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.3">
@@ -2883,10 +2883,10 @@
         <v>9</v>
       </c>
       <c r="B223">
-        <v>1871</v>
+        <v>1456</v>
       </c>
       <c r="C223">
-        <v>51581.270062155127</v>
+        <v>51425.245286726502</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.3">
@@ -2894,10 +2894,10 @@
         <v>9</v>
       </c>
       <c r="B224">
-        <v>2413</v>
+        <v>1871</v>
       </c>
       <c r="C224">
-        <v>51927.463843974918</v>
+        <v>51581.270062155127</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.3">
@@ -2905,10 +2905,10 @@
         <v>9</v>
       </c>
       <c r="B225">
-        <v>2574</v>
+        <v>2413</v>
       </c>
       <c r="C225">
-        <v>56780.625213898224</v>
+        <v>51927.463843974918</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.3">
@@ -2916,10 +2916,10 @@
         <v>9</v>
       </c>
       <c r="B226">
-        <v>2276</v>
+        <v>2574</v>
       </c>
       <c r="C226">
-        <v>63903.473762958361</v>
+        <v>56780.625213898224</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.3">
@@ -2927,10 +2927,10 @@
         <v>9</v>
       </c>
       <c r="B227">
-        <v>2705</v>
+        <v>2276</v>
       </c>
       <c r="C227">
-        <v>67682.54798142401</v>
+        <v>63903.473762958361</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.3">
@@ -2938,10 +2938,10 @@
         <v>9</v>
       </c>
       <c r="B228">
-        <v>2546</v>
+        <v>2705</v>
       </c>
       <c r="C228">
-        <v>1512.6094425225172</v>
+        <v>67682.54798142401</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.3">
@@ -2949,10 +2949,10 @@
         <v>9</v>
       </c>
       <c r="B229">
-        <v>2547</v>
+        <v>2546</v>
       </c>
       <c r="C229">
-        <v>13804.888899292078</v>
+        <v>1512.6094425225172</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.3">
@@ -2960,10 +2960,10 @@
         <v>9</v>
       </c>
       <c r="B230">
-        <v>2549</v>
+        <v>2547</v>
       </c>
       <c r="C230">
-        <v>7739.5339892319562</v>
+        <v>13804.888899292078</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.3">
@@ -2971,10 +2971,10 @@
         <v>9</v>
       </c>
       <c r="B231">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="C231">
-        <v>10266.443523665548</v>
+        <v>7739.5339892319562</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.3">
@@ -2982,10 +2982,10 @@
         <v>9</v>
       </c>
       <c r="B232">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="C232">
-        <v>8758.1206071851193</v>
+        <v>10266.443523665548</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.3">
@@ -2993,10 +2993,10 @@
         <v>9</v>
       </c>
       <c r="B233">
-        <v>2552</v>
+        <v>2551</v>
       </c>
       <c r="C233">
-        <v>27852.843761879078</v>
+        <v>8758.1206071851193</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.3">
@@ -3004,10 +3004,10 @@
         <v>9</v>
       </c>
       <c r="B234">
-        <v>2554</v>
+        <v>2552</v>
       </c>
       <c r="C234">
-        <v>6584.7069041752166</v>
+        <v>27852.843761879078</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.3">
@@ -3015,10 +3015,10 @@
         <v>9</v>
       </c>
       <c r="B235">
-        <v>2555</v>
+        <v>2554</v>
       </c>
       <c r="C235">
-        <v>14964.631105911165</v>
+        <v>6584.7069041752166</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.3">
@@ -3026,10 +3026,10 @@
         <v>9</v>
       </c>
       <c r="B236">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="C236">
-        <v>9355.0258993110856</v>
+        <v>14964.631105911165</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.3">
@@ -3037,10 +3037,10 @@
         <v>9</v>
       </c>
       <c r="B237">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="C237">
-        <v>14761.008874017321</v>
+        <v>9355.0258993110856</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.3">
@@ -3048,10 +3048,10 @@
         <v>9</v>
       </c>
       <c r="B238">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="C238">
-        <v>15520.892511574631</v>
+        <v>14761.008874017321</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.3">
@@ -3059,10 +3059,10 @@
         <v>9</v>
       </c>
       <c r="B239">
-        <v>2561</v>
+        <v>2558</v>
       </c>
       <c r="C239">
-        <v>365.83795081160144</v>
+        <v>15520.892511574631</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.3">
@@ -3070,10 +3070,10 @@
         <v>9</v>
       </c>
       <c r="B240">
-        <v>2562</v>
+        <v>2561</v>
       </c>
       <c r="C240">
-        <v>5810.54295767247</v>
+        <v>365.83795081160144</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.3">
@@ -3081,10 +3081,10 @@
         <v>9</v>
       </c>
       <c r="B241">
-        <v>2249</v>
+        <v>2562</v>
       </c>
       <c r="C241">
-        <v>68980.559971745941</v>
+        <v>5810.54295767247</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.3">
@@ -3092,10 +3092,10 @@
         <v>9</v>
       </c>
       <c r="B242">
-        <v>2146</v>
+        <v>2249</v>
       </c>
       <c r="C242">
-        <v>72929.553826811418</v>
+        <v>68980.559971745941</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.3">
@@ -3103,10 +3103,10 @@
         <v>9</v>
       </c>
       <c r="B243">
-        <v>1450</v>
+        <v>2146</v>
       </c>
       <c r="C243">
-        <v>73560.72588553559</v>
+        <v>72929.553826811418</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.3">
@@ -3114,10 +3114,10 @@
         <v>9</v>
       </c>
       <c r="B244">
-        <v>1142</v>
+        <v>1450</v>
       </c>
       <c r="C244">
-        <v>92432.999168746464</v>
+        <v>73560.72588553559</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.3">
@@ -3125,10 +3125,10 @@
         <v>9</v>
       </c>
       <c r="B245">
-        <v>2541</v>
+        <v>1142</v>
       </c>
       <c r="C245">
-        <v>115888.88600630446</v>
+        <v>92432.999168746464</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.3">
@@ -3136,10 +3136,10 @@
         <v>9</v>
       </c>
       <c r="B246">
-        <v>2627</v>
+        <v>2541</v>
       </c>
       <c r="C246">
-        <v>6164.4017752889076</v>
+        <v>115888.88600630446</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.3">
@@ -3147,10 +3147,10 @@
         <v>9</v>
       </c>
       <c r="B247">
-        <v>2510</v>
+        <v>2627</v>
       </c>
       <c r="C247">
-        <v>121564.03775893</v>
+        <v>6164.4017752889076</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.3">
@@ -3158,21 +3158,21 @@
         <v>9</v>
       </c>
       <c r="B248">
+        <v>2510</v>
+      </c>
+      <c r="C248">
+        <v>121564.03775893</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A249">
+        <v>9</v>
+      </c>
+      <c r="B249">
         <v>1907</v>
       </c>
-      <c r="C248">
+      <c r="C249">
         <v>150261.31219061578</v>
-      </c>
-    </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A249" t="s">
-        <v>3</v>
-      </c>
-      <c r="B249">
-        <v>569</v>
-      </c>
-      <c r="C249">
-        <v>567637.70997093734</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.3">
@@ -3180,10 +3180,10 @@
         <v>3</v>
       </c>
       <c r="B250">
-        <v>1317</v>
+        <v>569</v>
       </c>
       <c r="C250">
-        <v>52466.505623578487</v>
+        <v>567637.70997093734</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.3">
@@ -3191,10 +3191,10 @@
         <v>3</v>
       </c>
       <c r="B251">
-        <v>353</v>
+        <v>1317</v>
       </c>
       <c r="C251">
-        <v>49002.621259188832</v>
+        <v>52466.505623578487</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.3">
@@ -3202,10 +3202,10 @@
         <v>3</v>
       </c>
       <c r="B252">
-        <v>1289</v>
+        <v>353</v>
       </c>
       <c r="C252">
-        <v>43687.879397867531</v>
+        <v>49002.621259188832</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.3">
@@ -3213,10 +3213,10 @@
         <v>3</v>
       </c>
       <c r="B253">
-        <v>2660</v>
+        <v>1289</v>
       </c>
       <c r="C253">
-        <v>40183.849616796331</v>
+        <v>43687.879397867531</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.3">
@@ -3224,10 +3224,10 @@
         <v>3</v>
       </c>
       <c r="B254">
-        <v>2197</v>
+        <v>2660</v>
       </c>
       <c r="C254">
-        <v>36044.136301060404</v>
+        <v>40183.849616796331</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.3">
@@ -3235,10 +3235,10 @@
         <v>3</v>
       </c>
       <c r="B255">
-        <v>525</v>
+        <v>2197</v>
       </c>
       <c r="C255">
-        <v>35950.768052918022</v>
+        <v>36044.136301060404</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.3">
@@ -3246,10 +3246,10 @@
         <v>3</v>
       </c>
       <c r="B256">
-        <v>1956</v>
+        <v>525</v>
       </c>
       <c r="C256">
-        <v>34038.081085334641</v>
+        <v>35950.768052918022</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.3">
@@ -3257,10 +3257,10 @@
         <v>3</v>
       </c>
       <c r="B257">
-        <v>941</v>
+        <v>1956</v>
       </c>
       <c r="C257">
-        <v>32747.166564230884</v>
+        <v>34038.081085334641</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.3">
@@ -3268,10 +3268,10 @@
         <v>3</v>
       </c>
       <c r="B258">
-        <v>1632</v>
+        <v>941</v>
       </c>
       <c r="C258">
-        <v>31684.800026177258</v>
+        <v>32747.166564230884</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.3">
@@ -3279,10 +3279,10 @@
         <v>3</v>
       </c>
       <c r="B259">
-        <v>1890</v>
+        <v>1632</v>
       </c>
       <c r="C259">
-        <v>30754.807986715925</v>
+        <v>31684.800026177258</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.3">
@@ -3290,10 +3290,10 @@
         <v>3</v>
       </c>
       <c r="B260">
-        <v>767</v>
+        <v>1890</v>
       </c>
       <c r="C260">
-        <v>29163.436807875081</v>
+        <v>30754.807986715925</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.3">
@@ -3301,10 +3301,10 @@
         <v>3</v>
       </c>
       <c r="B261">
-        <v>609</v>
+        <v>767</v>
       </c>
       <c r="C261">
-        <v>27945.835198973171</v>
+        <v>29163.436807875081</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.3">
@@ -3312,10 +3312,10 @@
         <v>3</v>
       </c>
       <c r="B262">
-        <v>1254</v>
+        <v>609</v>
       </c>
       <c r="C262">
-        <v>24794.497610100807</v>
+        <v>27945.835198973171</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.3">
@@ -3323,10 +3323,10 @@
         <v>3</v>
       </c>
       <c r="B263">
-        <v>947</v>
+        <v>1254</v>
       </c>
       <c r="C263">
-        <v>21914.076073917324</v>
+        <v>24794.497610100807</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.3">
@@ -3334,10 +3334,10 @@
         <v>3</v>
       </c>
       <c r="B264">
-        <v>2773</v>
+        <v>947</v>
       </c>
       <c r="C264">
-        <v>19828.314865954195</v>
+        <v>21914.076073917324</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.3">
@@ -3345,10 +3345,10 @@
         <v>3</v>
       </c>
       <c r="B265">
-        <v>2026</v>
+        <v>2773</v>
       </c>
       <c r="C265">
-        <v>19426.273542132072</v>
+        <v>19828.314865954195</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.3">
@@ -3356,10 +3356,10 @@
         <v>3</v>
       </c>
       <c r="B266">
-        <v>2686</v>
+        <v>2026</v>
       </c>
       <c r="C266">
-        <v>19139.920534510304</v>
+        <v>19426.273542132072</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.3">
@@ -3367,10 +3367,10 @@
         <v>3</v>
       </c>
       <c r="B267">
-        <v>2769</v>
+        <v>2686</v>
       </c>
       <c r="C267">
-        <v>18096.592580705241</v>
+        <v>19139.920534510304</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.3">
@@ -3378,10 +3378,10 @@
         <v>3</v>
       </c>
       <c r="B268">
-        <v>2657</v>
+        <v>2769</v>
       </c>
       <c r="C268">
-        <v>17438.79463421469</v>
+        <v>18096.592580705241</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.3">
@@ -3389,10 +3389,10 @@
         <v>3</v>
       </c>
       <c r="B269">
-        <v>2648</v>
+        <v>2657</v>
       </c>
       <c r="C269">
-        <v>17377.017809574252</v>
+        <v>17438.79463421469</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.3">
@@ -3400,10 +3400,10 @@
         <v>3</v>
       </c>
       <c r="B270">
-        <v>2787</v>
+        <v>2648</v>
       </c>
       <c r="C270">
-        <v>17063.477831944059</v>
+        <v>17377.017809574252</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.3">
@@ -3411,10 +3411,10 @@
         <v>3</v>
       </c>
       <c r="B271">
-        <v>2789</v>
+        <v>2787</v>
       </c>
       <c r="C271">
-        <v>16276.242188745029</v>
+        <v>17063.477831944059</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.3">
@@ -3422,10 +3422,10 @@
         <v>3</v>
       </c>
       <c r="B272">
-        <v>2682</v>
+        <v>2789</v>
       </c>
       <c r="C272">
-        <v>15801.542296723319</v>
+        <v>16276.242188745029</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.3">
@@ -3433,10 +3433,10 @@
         <v>3</v>
       </c>
       <c r="B273">
-        <v>2528</v>
+        <v>2682</v>
       </c>
       <c r="C273">
-        <v>15732.774105521043</v>
+        <v>15801.542296723319</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.3">
@@ -3444,10 +3444,10 @@
         <v>3</v>
       </c>
       <c r="B274">
-        <v>931</v>
+        <v>2528</v>
       </c>
       <c r="C274">
-        <v>15655.317272871356</v>
+        <v>15732.774105521043</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.3">
@@ -3455,10 +3455,10 @@
         <v>3</v>
       </c>
       <c r="B275">
-        <v>2726</v>
+        <v>931</v>
       </c>
       <c r="C275">
-        <v>15550.117807784596</v>
+        <v>15655.317272871356</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.3">
@@ -3466,10 +3466,10 @@
         <v>3</v>
       </c>
       <c r="B276">
-        <v>2667</v>
+        <v>2726</v>
       </c>
       <c r="C276">
-        <v>15000</v>
+        <v>15550.117807784596</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.3">
@@ -3477,7 +3477,7 @@
         <v>3</v>
       </c>
       <c r="B277">
-        <v>2810</v>
+        <v>2667</v>
       </c>
       <c r="C277">
         <v>15000</v>
@@ -3488,7 +3488,7 @@
         <v>3</v>
       </c>
       <c r="B278">
-        <v>2791</v>
+        <v>2810</v>
       </c>
       <c r="C278">
         <v>15000</v>
@@ -3499,7 +3499,7 @@
         <v>3</v>
       </c>
       <c r="B279">
-        <v>2045</v>
+        <v>2791</v>
       </c>
       <c r="C279">
         <v>15000</v>
@@ -3510,7 +3510,7 @@
         <v>3</v>
       </c>
       <c r="B280">
-        <v>1076</v>
+        <v>2045</v>
       </c>
       <c r="C280">
         <v>15000</v>
@@ -3521,7 +3521,7 @@
         <v>3</v>
       </c>
       <c r="B281">
-        <v>2760</v>
+        <v>1076</v>
       </c>
       <c r="C281">
         <v>15000</v>
@@ -3532,7 +3532,7 @@
         <v>3</v>
       </c>
       <c r="B282">
-        <v>2790</v>
+        <v>2760</v>
       </c>
       <c r="C282">
         <v>15000</v>
@@ -3543,7 +3543,7 @@
         <v>3</v>
       </c>
       <c r="B283">
-        <v>2801</v>
+        <v>2790</v>
       </c>
       <c r="C283">
         <v>15000</v>
@@ -3554,7 +3554,7 @@
         <v>3</v>
       </c>
       <c r="B284">
-        <v>2580</v>
+        <v>2801</v>
       </c>
       <c r="C284">
         <v>15000</v>
@@ -3565,7 +3565,7 @@
         <v>3</v>
       </c>
       <c r="B285">
-        <v>2708</v>
+        <v>2580</v>
       </c>
       <c r="C285">
         <v>15000</v>
@@ -3576,7 +3576,7 @@
         <v>3</v>
       </c>
       <c r="B286">
-        <v>2019</v>
+        <v>2708</v>
       </c>
       <c r="C286">
         <v>15000</v>
@@ -3587,7 +3587,7 @@
         <v>3</v>
       </c>
       <c r="B287">
-        <v>2641</v>
+        <v>2019</v>
       </c>
       <c r="C287">
         <v>15000</v>
@@ -3598,7 +3598,7 @@
         <v>3</v>
       </c>
       <c r="B288">
-        <v>2711</v>
+        <v>2641</v>
       </c>
       <c r="C288">
         <v>15000</v>
@@ -3609,7 +3609,7 @@
         <v>3</v>
       </c>
       <c r="B289">
-        <v>2516</v>
+        <v>2711</v>
       </c>
       <c r="C289">
         <v>15000</v>
@@ -3620,7 +3620,7 @@
         <v>3</v>
       </c>
       <c r="B290">
-        <v>2577</v>
+        <v>2516</v>
       </c>
       <c r="C290">
         <v>15000</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="B291">
-        <v>1846</v>
+        <v>2577</v>
       </c>
       <c r="C291">
         <v>15000</v>
@@ -3642,7 +3642,7 @@
         <v>3</v>
       </c>
       <c r="B292">
-        <v>2639</v>
+        <v>1846</v>
       </c>
       <c r="C292">
         <v>15000</v>
@@ -3653,7 +3653,7 @@
         <v>3</v>
       </c>
       <c r="B293">
-        <v>2472</v>
+        <v>2639</v>
       </c>
       <c r="C293">
         <v>15000</v>
@@ -3664,7 +3664,7 @@
         <v>3</v>
       </c>
       <c r="B294">
-        <v>2687</v>
+        <v>2472</v>
       </c>
       <c r="C294">
         <v>15000</v>
@@ -3675,7 +3675,7 @@
         <v>3</v>
       </c>
       <c r="B295">
-        <v>2730</v>
+        <v>2687</v>
       </c>
       <c r="C295">
         <v>15000</v>
@@ -3686,7 +3686,7 @@
         <v>3</v>
       </c>
       <c r="B296">
-        <v>2728</v>
+        <v>2730</v>
       </c>
       <c r="C296">
         <v>15000</v>
@@ -3697,7 +3697,7 @@
         <v>3</v>
       </c>
       <c r="B297">
-        <v>2607</v>
+        <v>2728</v>
       </c>
       <c r="C297">
         <v>15000</v>
@@ -3708,7 +3708,7 @@
         <v>3</v>
       </c>
       <c r="B298">
-        <v>2793</v>
+        <v>2607</v>
       </c>
       <c r="C298">
         <v>15000</v>
@@ -3719,10 +3719,10 @@
         <v>3</v>
       </c>
       <c r="B299">
-        <v>2582</v>
+        <v>2793</v>
       </c>
       <c r="C299">
-        <v>9124.8426649896664</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.3">
@@ -3730,10 +3730,10 @@
         <v>3</v>
       </c>
       <c r="B300">
-        <v>2345</v>
+        <v>2582</v>
       </c>
       <c r="C300">
-        <v>9000.1825689196139</v>
+        <v>9124.8426649896664</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.3">
@@ -3741,10 +3741,10 @@
         <v>3</v>
       </c>
       <c r="B301">
-        <v>630</v>
+        <v>2345</v>
       </c>
       <c r="C301">
-        <v>7602.5075159437756</v>
+        <v>9000.1825689196139</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.3">
@@ -3752,10 +3752,10 @@
         <v>3</v>
       </c>
       <c r="B302">
-        <v>2216</v>
+        <v>630</v>
       </c>
       <c r="C302">
-        <v>7095.2014819442547</v>
+        <v>7602.5075159437756</v>
       </c>
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.3">
@@ -3763,10 +3763,10 @@
         <v>3</v>
       </c>
       <c r="B303">
-        <v>925</v>
+        <v>2216</v>
       </c>
       <c r="C303">
-        <v>6335.1999712518345</v>
+        <v>7095.2014819442547</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.3">
@@ -3774,10 +3774,10 @@
         <v>3</v>
       </c>
       <c r="B304">
-        <v>2716</v>
+        <v>925</v>
       </c>
       <c r="C304">
-        <v>4946.7782472310919</v>
+        <v>6335.1999712518345</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.3">
@@ -3785,10 +3785,10 @@
         <v>3</v>
       </c>
       <c r="B305">
-        <v>374</v>
+        <v>2716</v>
       </c>
       <c r="C305">
-        <v>3711.0283082092114</v>
+        <v>4946.7782472310919</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.3">
@@ -3796,10 +3796,10 @@
         <v>3</v>
       </c>
       <c r="B306">
-        <v>2637</v>
+        <v>374</v>
       </c>
       <c r="C306">
-        <v>3344.9707691720714</v>
+        <v>3711.0283082092114</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.3">
@@ -3807,10 +3807,10 @@
         <v>3</v>
       </c>
       <c r="B307">
-        <v>2584</v>
+        <v>2637</v>
       </c>
       <c r="C307">
-        <v>2789.6085880483056</v>
+        <v>3344.9707691720714</v>
       </c>
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.3">
@@ -3818,10 +3818,10 @@
         <v>3</v>
       </c>
       <c r="B308">
-        <v>2689</v>
+        <v>2584</v>
       </c>
       <c r="C308">
-        <v>1710.4775791271645</v>
+        <v>2789.6085880483056</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.3">
@@ -3829,10 +3829,10 @@
         <v>3</v>
       </c>
       <c r="B309">
-        <v>2734</v>
+        <v>2689</v>
       </c>
       <c r="C309">
-        <v>940.4150223832753</v>
+        <v>1710.4775791271645</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.3">
@@ -3840,10 +3840,10 @@
         <v>3</v>
       </c>
       <c r="B310">
-        <v>325</v>
+        <v>2734</v>
       </c>
       <c r="C310">
-        <v>894.58125407365185</v>
+        <v>940.4150223832753</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.3">
@@ -3851,10 +3851,10 @@
         <v>3</v>
       </c>
       <c r="B311">
-        <v>562</v>
+        <v>325</v>
       </c>
       <c r="C311">
-        <v>863.87933668693267</v>
+        <v>894.58125407365185</v>
       </c>
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.3">
@@ -3862,10 +3862,10 @@
         <v>3</v>
       </c>
       <c r="B312">
-        <v>2802</v>
+        <v>562</v>
       </c>
       <c r="C312">
-        <v>596.06703896986335</v>
+        <v>863.87933668693267</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.3">
@@ -3873,10 +3873,10 @@
         <v>3</v>
       </c>
       <c r="B313">
-        <v>1840</v>
+        <v>2802</v>
       </c>
       <c r="C313">
-        <v>415.09743533486176</v>
+        <v>596.06703896986335</v>
       </c>
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.3">
@@ -3884,10 +3884,10 @@
         <v>3</v>
       </c>
       <c r="B314">
-        <v>2715</v>
+        <v>1840</v>
       </c>
       <c r="C314">
-        <v>217.59190241117861</v>
+        <v>415.09743533486176</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.3">
@@ -3895,21 +3895,21 @@
         <v>3</v>
       </c>
       <c r="B315">
-        <v>11</v>
+        <v>2715</v>
       </c>
       <c r="C315">
-        <v>-253.16065053843562</v>
+        <v>217.59190241117861</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B316">
-        <v>325</v>
+        <v>11</v>
       </c>
       <c r="C316">
-        <v>1823.8679890494018</v>
+        <v>-253.16065053843562</v>
       </c>
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.3">
@@ -3917,10 +3917,10 @@
         <v>4</v>
       </c>
       <c r="B317">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C317">
-        <v>902.8488102721501</v>
+        <v>1823.8679890494018</v>
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.3">
@@ -3928,10 +3928,10 @@
         <v>4</v>
       </c>
       <c r="B318">
-        <v>358</v>
+        <v>326</v>
       </c>
       <c r="C318">
-        <v>77156.847182285579</v>
+        <v>902.8488102721501</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.3">
@@ -3939,10 +3939,10 @@
         <v>4</v>
       </c>
       <c r="B319">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C319">
-        <v>141470.97</v>
+        <v>77156.847182285579</v>
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.3">
@@ -3950,10 +3950,10 @@
         <v>4</v>
       </c>
       <c r="B320">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C320">
-        <v>76564.066916899654</v>
+        <v>141470.97</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.3">
@@ -3961,10 +3961,10 @@
         <v>4</v>
       </c>
       <c r="B321">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="C321">
-        <v>1759.3344302732141</v>
+        <v>76564.066916899654</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.3">
@@ -3972,10 +3972,10 @@
         <v>4</v>
       </c>
       <c r="B322">
-        <v>429</v>
+        <v>374</v>
       </c>
       <c r="C322">
-        <v>47099.4</v>
+        <v>1759.3344302732141</v>
       </c>
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.3">
@@ -3983,10 +3983,10 @@
         <v>4</v>
       </c>
       <c r="B323">
-        <v>535</v>
+        <v>429</v>
       </c>
       <c r="C323">
-        <v>72475.414579673743</v>
+        <v>47099.4</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.3">
@@ -3994,10 +3994,10 @@
         <v>4</v>
       </c>
       <c r="B324">
-        <v>626</v>
+        <v>535</v>
       </c>
       <c r="C324">
-        <v>387451.76227699558</v>
+        <v>72475.414579673743</v>
       </c>
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.3">
@@ -4005,10 +4005,10 @@
         <v>4</v>
       </c>
       <c r="B325">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C325">
-        <v>14027.334732089985</v>
+        <v>387451.76227699558</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.3">
@@ -4016,10 +4016,10 @@
         <v>4</v>
       </c>
       <c r="B326">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="C326">
-        <v>40218.51</v>
+        <v>14027.334732089985</v>
       </c>
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.3">
@@ -4027,10 +4027,10 @@
         <v>4</v>
       </c>
       <c r="B327">
-        <v>675</v>
+        <v>636</v>
       </c>
       <c r="C327">
-        <v>33447.636574796554</v>
+        <v>40218.51</v>
       </c>
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.3">
@@ -4038,10 +4038,10 @@
         <v>4</v>
       </c>
       <c r="B328">
-        <v>692</v>
+        <v>675</v>
       </c>
       <c r="C328">
-        <v>0</v>
+        <v>33447.636574796554</v>
       </c>
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.3">
@@ -4049,10 +4049,10 @@
         <v>4</v>
       </c>
       <c r="B329">
-        <v>945</v>
+        <v>692</v>
       </c>
       <c r="C329">
-        <v>34453.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.3">
@@ -4060,10 +4060,10 @@
         <v>4</v>
       </c>
       <c r="B330">
-        <v>1045</v>
+        <v>945</v>
       </c>
       <c r="C330">
-        <v>15000</v>
+        <v>34453.4</v>
       </c>
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.3">
@@ -4071,10 +4071,10 @@
         <v>4</v>
       </c>
       <c r="B331">
-        <v>1108</v>
+        <v>1045</v>
       </c>
       <c r="C331">
-        <v>31308.056694668532</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.3">
@@ -4082,10 +4082,10 @@
         <v>4</v>
       </c>
       <c r="B332">
-        <v>1137</v>
+        <v>1108</v>
       </c>
       <c r="C332">
-        <v>196060.36</v>
+        <v>31308.056694668532</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.3">
@@ -4093,10 +4093,10 @@
         <v>4</v>
       </c>
       <c r="B333">
-        <v>1261</v>
+        <v>1137</v>
       </c>
       <c r="C333">
-        <v>38802.85069322717</v>
+        <v>196060.36</v>
       </c>
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.3">
@@ -4104,10 +4104,10 @@
         <v>4</v>
       </c>
       <c r="B334">
-        <v>1293</v>
+        <v>1261</v>
       </c>
       <c r="C334">
-        <v>100272.94</v>
+        <v>38802.85069322717</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.3">
@@ -4115,10 +4115,10 @@
         <v>4</v>
       </c>
       <c r="B335">
-        <v>1308</v>
+        <v>1293</v>
       </c>
       <c r="C335">
-        <v>33712.998706487044</v>
+        <v>100272.94</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.3">
@@ -4126,10 +4126,10 @@
         <v>4</v>
       </c>
       <c r="B336">
-        <v>1392</v>
+        <v>1308</v>
       </c>
       <c r="C336">
-        <v>3853.8212846225574</v>
+        <v>33712.998706487044</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.3">
@@ -4137,10 +4137,10 @@
         <v>4</v>
       </c>
       <c r="B337">
-        <v>1653</v>
+        <v>1392</v>
       </c>
       <c r="C337">
-        <v>77383.811874679785</v>
+        <v>3853.8212846225574</v>
       </c>
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.3">
@@ -4148,10 +4148,10 @@
         <v>4</v>
       </c>
       <c r="B338">
-        <v>1823</v>
+        <v>1653</v>
       </c>
       <c r="C338">
-        <v>15000</v>
+        <v>77383.811874679785</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.3">
@@ -4159,10 +4159,10 @@
         <v>4</v>
       </c>
       <c r="B339">
-        <v>1906</v>
+        <v>1823</v>
       </c>
       <c r="C339">
-        <v>21140.587231043661</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.3">
@@ -4170,10 +4170,10 @@
         <v>4</v>
       </c>
       <c r="B340">
-        <v>2015</v>
+        <v>1906</v>
       </c>
       <c r="C340">
-        <v>58214.98162022305</v>
+        <v>21140.587231043661</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.3">
@@ -4181,10 +4181,10 @@
         <v>4</v>
       </c>
       <c r="B341">
-        <v>2107</v>
+        <v>2015</v>
       </c>
       <c r="C341">
-        <v>109621.02424363823</v>
+        <v>58214.98162022305</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.3">
@@ -4192,10 +4192,10 @@
         <v>4</v>
       </c>
       <c r="B342">
-        <v>2109</v>
+        <v>2107</v>
       </c>
       <c r="C342">
-        <v>15000</v>
+        <v>109621.02424363823</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.3">
@@ -4203,10 +4203,10 @@
         <v>4</v>
       </c>
       <c r="B343">
-        <v>2114</v>
+        <v>2109</v>
       </c>
       <c r="C343">
-        <v>16352.689379832818</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.3">
@@ -4214,10 +4214,10 @@
         <v>4</v>
       </c>
       <c r="B344">
-        <v>2118</v>
+        <v>2114</v>
       </c>
       <c r="C344">
-        <v>69687.832795976705</v>
+        <v>16352.689379832818</v>
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.3">
@@ -4225,10 +4225,10 @@
         <v>4</v>
       </c>
       <c r="B345">
-        <v>2201</v>
+        <v>2118</v>
       </c>
       <c r="C345">
-        <v>204.97440699409825</v>
+        <v>69687.832795976705</v>
       </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.3">
@@ -4236,10 +4236,10 @@
         <v>4</v>
       </c>
       <c r="B346">
-        <v>2211</v>
+        <v>2201</v>
       </c>
       <c r="C346">
-        <v>74015.535398273918</v>
+        <v>204.97440699409825</v>
       </c>
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.3">
@@ -4247,10 +4247,10 @@
         <v>4</v>
       </c>
       <c r="B347">
-        <v>2308</v>
+        <v>2211</v>
       </c>
       <c r="C347">
-        <v>27283.948571802139</v>
+        <v>74015.535398273918</v>
       </c>
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.3">
@@ -4258,10 +4258,10 @@
         <v>4</v>
       </c>
       <c r="B348">
-        <v>2330</v>
+        <v>2308</v>
       </c>
       <c r="C348">
-        <v>15000</v>
+        <v>27283.948571802139</v>
       </c>
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.3">
@@ -4269,10 +4269,10 @@
         <v>4</v>
       </c>
       <c r="B349">
-        <v>2359</v>
+        <v>2330</v>
       </c>
       <c r="C349">
-        <v>17115.396352551164</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="350" spans="1:3" x14ac:dyDescent="0.3">
@@ -4280,10 +4280,10 @@
         <v>4</v>
       </c>
       <c r="B350">
-        <v>2366</v>
+        <v>2359</v>
       </c>
       <c r="C350">
-        <v>15000</v>
+        <v>17115.396352551164</v>
       </c>
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.3">
@@ -4291,10 +4291,10 @@
         <v>4</v>
       </c>
       <c r="B351">
-        <v>2383</v>
+        <v>2366</v>
       </c>
       <c r="C351">
-        <v>25236.019576771883</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.3">
@@ -4302,10 +4302,10 @@
         <v>4</v>
       </c>
       <c r="B352">
-        <v>2491</v>
+        <v>2383</v>
       </c>
       <c r="C352">
-        <v>15708.103307654304</v>
+        <v>25236.019576771883</v>
       </c>
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.3">
@@ -4313,10 +4313,10 @@
         <v>4</v>
       </c>
       <c r="B353">
-        <v>2507</v>
+        <v>2491</v>
       </c>
       <c r="C353">
-        <v>15000</v>
+        <v>15708.103307654304</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.3">
@@ -4324,7 +4324,7 @@
         <v>4</v>
       </c>
       <c r="B354">
-        <v>2530</v>
+        <v>2507</v>
       </c>
       <c r="C354">
         <v>15000</v>
@@ -4335,7 +4335,7 @@
         <v>4</v>
       </c>
       <c r="B355">
-        <v>2571</v>
+        <v>2530</v>
       </c>
       <c r="C355">
         <v>15000</v>
@@ -4346,7 +4346,7 @@
         <v>4</v>
       </c>
       <c r="B356">
-        <v>2576</v>
+        <v>2571</v>
       </c>
       <c r="C356">
         <v>15000</v>
@@ -4357,7 +4357,7 @@
         <v>4</v>
       </c>
       <c r="B357">
-        <v>2678</v>
+        <v>2576</v>
       </c>
       <c r="C357">
         <v>15000</v>
@@ -4368,10 +4368,10 @@
         <v>4</v>
       </c>
       <c r="B358">
-        <v>2680</v>
+        <v>2678</v>
       </c>
       <c r="C358">
-        <v>17653.191516466668</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.3">
@@ -4379,10 +4379,10 @@
         <v>4</v>
       </c>
       <c r="B359">
-        <v>2681</v>
+        <v>2680</v>
       </c>
       <c r="C359">
-        <v>18087.411572689049</v>
+        <v>17653.191516466668</v>
       </c>
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.3">
@@ -4390,10 +4390,10 @@
         <v>4</v>
       </c>
       <c r="B360">
-        <v>2691</v>
+        <v>2681</v>
       </c>
       <c r="C360">
-        <v>30743.31</v>
+        <v>18087.411572689049</v>
       </c>
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.3">
@@ -4401,10 +4401,10 @@
         <v>4</v>
       </c>
       <c r="B361">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="C361">
-        <v>15000</v>
+        <v>30743.31</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.3">
@@ -4412,10 +4412,10 @@
         <v>4</v>
       </c>
       <c r="B362">
-        <v>2696</v>
+        <v>2692</v>
       </c>
       <c r="C362">
-        <v>68173.211828627595</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.3">
@@ -4423,10 +4423,10 @@
         <v>4</v>
       </c>
       <c r="B363">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="C363">
-        <v>27058.895143994421</v>
+        <v>68173.211828627595</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.3">
@@ -4434,10 +4434,10 @@
         <v>4</v>
       </c>
       <c r="B364">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="C364">
-        <v>21540.450340488205</v>
+        <v>27058.895143994421</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.3">
@@ -4445,10 +4445,10 @@
         <v>4</v>
       </c>
       <c r="B365">
-        <v>2709</v>
+        <v>2698</v>
       </c>
       <c r="C365">
-        <v>29749.635377291357</v>
+        <v>21540.450340488205</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.3">
@@ -4456,10 +4456,10 @@
         <v>4</v>
       </c>
       <c r="B366">
-        <v>2716</v>
+        <v>2709</v>
       </c>
       <c r="C366">
-        <v>2743.3058857573801</v>
+        <v>29749.635377291357</v>
       </c>
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.3">
@@ -4467,10 +4467,10 @@
         <v>4</v>
       </c>
       <c r="B367">
-        <v>2755</v>
+        <v>2716</v>
       </c>
       <c r="C367">
-        <v>15204.97</v>
+        <v>2743.3058857573801</v>
       </c>
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.3">
@@ -4478,10 +4478,10 @@
         <v>4</v>
       </c>
       <c r="B368">
-        <v>2767</v>
+        <v>2755</v>
       </c>
       <c r="C368">
-        <v>21589.803591399374</v>
+        <v>15204.97</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.3">
@@ -4489,10 +4489,10 @@
         <v>4</v>
       </c>
       <c r="B369">
-        <v>2768</v>
+        <v>2767</v>
       </c>
       <c r="C369">
-        <v>74786.275879616267</v>
+        <v>21589.803591399374</v>
       </c>
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.3">
@@ -4500,9 +4500,20 @@
         <v>4</v>
       </c>
       <c r="B370">
+        <v>2768</v>
+      </c>
+      <c r="C370">
+        <v>74786.275879616267</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A371" t="s">
+        <v>4</v>
+      </c>
+      <c r="B371">
         <v>2799</v>
       </c>
-      <c r="C370">
+      <c r="C371">
         <v>15000</v>
       </c>
     </row>

</xml_diff>